<commit_message>
Map keys label boundaries so they fit a phone; translations for every changed sentence; rebuilt workbooks
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FWx24PCx3Jw4SUDQC6oU7o
</commit_message>
<xml_diff>
--- a/downloads/gujarat.xlsx
+++ b/downloads/gujarat.xlsx
@@ -801,7 +801,7 @@
         <v>30259</v>
       </c>
       <c r="F2" t="n">
-        <v>11.53</v>
+        <v>11.5269</v>
       </c>
       <c r="G2" t="n">
         <v>8050</v>
@@ -822,7 +822,7 @@
         <v>232248</v>
       </c>
       <c r="M2" t="n">
-        <v>-1.14</v>
+        <v>-1.1418</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -864,7 +864,7 @@
         <v>27824</v>
       </c>
       <c r="F3" t="n">
-        <v>10.44</v>
+        <v>10.4442</v>
       </c>
       <c r="G3" t="n">
         <v>7639</v>
@@ -885,7 +885,7 @@
         <v>238581</v>
       </c>
       <c r="M3" t="n">
-        <v>-2.23</v>
+        <v>-2.2245</v>
       </c>
       <c r="N3" t="inlineStr">
         <is>
@@ -927,7 +927,7 @@
         <v>32682</v>
       </c>
       <c r="F4" t="n">
-        <v>10.69</v>
+        <v>10.6881</v>
       </c>
       <c r="G4" t="n">
         <v>11883</v>
@@ -948,7 +948,7 @@
         <v>273098</v>
       </c>
       <c r="M4" t="n">
-        <v>-1.98</v>
+        <v>-1.9806</v>
       </c>
       <c r="N4" t="inlineStr">
         <is>
@@ -990,7 +990,7 @@
         <v>39960</v>
       </c>
       <c r="F5" t="n">
-        <v>14.18</v>
+        <v>14.1783</v>
       </c>
       <c r="G5" t="n">
         <v>8343</v>
@@ -1011,7 +1011,7 @@
         <v>241879</v>
       </c>
       <c r="M5" t="n">
-        <v>1.51</v>
+        <v>1.5096</v>
       </c>
       <c r="N5" t="inlineStr">
         <is>
@@ -1053,7 +1053,7 @@
         <v>52176</v>
       </c>
       <c r="F6" t="n">
-        <v>16.41</v>
+        <v>16.4067</v>
       </c>
       <c r="G6" t="n">
         <v>10744</v>
@@ -1074,7 +1074,7 @@
         <v>265840</v>
       </c>
       <c r="M6" t="n">
-        <v>3.74</v>
+        <v>3.738</v>
       </c>
       <c r="N6" t="inlineStr">
         <is>
@@ -1116,7 +1116,7 @@
         <v>31274</v>
       </c>
       <c r="F7" t="n">
-        <v>12.21</v>
+        <v>12.2146</v>
       </c>
       <c r="G7" t="n">
         <v>8715</v>
@@ -1137,7 +1137,7 @@
         <v>224763</v>
       </c>
       <c r="M7" t="n">
-        <v>-0.46</v>
+        <v>-0.4541</v>
       </c>
       <c r="N7" t="inlineStr">
         <is>
@@ -1179,7 +1179,7 @@
         <v>18639</v>
       </c>
       <c r="F8" t="n">
-        <v>5.88</v>
+        <v>5.8792</v>
       </c>
       <c r="G8" t="n">
         <v>6310</v>
@@ -1200,7 +1200,7 @@
         <v>298393</v>
       </c>
       <c r="M8" t="n">
-        <v>-2.49</v>
+        <v>-2.4877</v>
       </c>
       <c r="N8" t="inlineStr">
         <is>
@@ -1242,7 +1242,7 @@
         <v>10762</v>
       </c>
       <c r="F9" t="n">
-        <v>4.07</v>
+        <v>4.0653</v>
       </c>
       <c r="G9" t="n">
         <v>4558</v>
@@ -1263,7 +1263,7 @@
         <v>253966</v>
       </c>
       <c r="M9" t="n">
-        <v>-4.3</v>
+        <v>-4.3016</v>
       </c>
       <c r="N9" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
         <v>20980</v>
       </c>
       <c r="F10" t="n">
-        <v>7.37</v>
+        <v>7.3705</v>
       </c>
       <c r="G10" t="n">
         <v>6595</v>
@@ -1326,7 +1326,7 @@
         <v>263667</v>
       </c>
       <c r="M10" t="n">
-        <v>-1</v>
+        <v>-0.9964</v>
       </c>
       <c r="N10" t="inlineStr">
         <is>
@@ -1368,7 +1368,7 @@
         <v>24667</v>
       </c>
       <c r="F11" t="n">
-        <v>9.01</v>
+        <v>9.0115</v>
       </c>
       <c r="G11" t="n">
         <v>7331</v>
@@ -1389,7 +1389,7 @@
         <v>249062</v>
       </c>
       <c r="M11" t="n">
-        <v>0.64</v>
+        <v>0.6446</v>
       </c>
       <c r="N11" t="inlineStr">
         <is>
@@ -1431,7 +1431,7 @@
         <v>29244</v>
       </c>
       <c r="F12" t="n">
-        <v>9.51</v>
+        <v>9.512499999999999</v>
       </c>
       <c r="G12" t="n">
         <v>8233</v>
@@ -1452,7 +1452,7 @@
         <v>278184</v>
       </c>
       <c r="M12" t="n">
-        <v>1.14</v>
+        <v>1.1456</v>
       </c>
       <c r="N12" t="inlineStr">
         <is>
@@ -1494,7 +1494,7 @@
         <v>40030</v>
       </c>
       <c r="F13" t="n">
-        <v>13.53</v>
+        <v>13.5312</v>
       </c>
       <c r="G13" t="n">
         <v>10912</v>
@@ -1515,7 +1515,7 @@
         <v>255805</v>
       </c>
       <c r="M13" t="n">
-        <v>5.16</v>
+        <v>5.1643</v>
       </c>
       <c r="N13" t="inlineStr">
         <is>
@@ -1557,7 +1557,7 @@
         <v>35464</v>
       </c>
       <c r="F14" t="n">
-        <v>11.58</v>
+        <v>11.578</v>
       </c>
       <c r="G14" t="n">
         <v>8619</v>
@@ -1578,7 +1578,7 @@
         <v>270841</v>
       </c>
       <c r="M14" t="n">
-        <v>3.21</v>
+        <v>3.2111</v>
       </c>
       <c r="N14" t="inlineStr">
         <is>
@@ -1620,7 +1620,7 @@
         <v>15876</v>
       </c>
       <c r="F15" t="n">
-        <v>5.98</v>
+        <v>5.9789</v>
       </c>
       <c r="G15" t="n">
         <v>5362</v>
@@ -1641,7 +1641,7 @@
         <v>249659</v>
       </c>
       <c r="M15" t="n">
-        <v>-2.39</v>
+        <v>-2.388</v>
       </c>
       <c r="N15" t="inlineStr">
         <is>
@@ -1683,7 +1683,7 @@
         <v>23965</v>
       </c>
       <c r="F16" t="n">
-        <v>7.74</v>
+        <v>7.7378</v>
       </c>
       <c r="G16" t="n">
         <v>7202</v>
@@ -1704,7 +1704,7 @@
         <v>285748</v>
       </c>
       <c r="M16" t="n">
-        <v>-0.63</v>
+        <v>-0.6291</v>
       </c>
       <c r="N16" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
         <v>27258</v>
       </c>
       <c r="F17" t="n">
-        <v>8.550000000000001</v>
+        <v>8.553100000000001</v>
       </c>
       <c r="G17" t="n">
         <v>5781</v>
@@ -1767,7 +1767,7 @@
         <v>291435</v>
       </c>
       <c r="M17" t="n">
-        <v>-0.26</v>
+        <v>-0.2539</v>
       </c>
       <c r="N17" t="inlineStr">
         <is>
@@ -1809,7 +1809,7 @@
         <v>19832</v>
       </c>
       <c r="F18" t="n">
-        <v>6.56</v>
+        <v>6.5634</v>
       </c>
       <c r="G18" t="n">
         <v>5813</v>
@@ -1830,7 +1830,7 @@
         <v>282328</v>
       </c>
       <c r="M18" t="n">
-        <v>-2.25</v>
+        <v>-2.2436</v>
       </c>
       <c r="N18" t="inlineStr">
         <is>
@@ -1872,7 +1872,7 @@
         <v>34884</v>
       </c>
       <c r="F19" t="n">
-        <v>10.99</v>
+        <v>10.9937</v>
       </c>
       <c r="G19" t="n">
         <v>7862</v>
@@ -1893,7 +1893,7 @@
         <v>282426</v>
       </c>
       <c r="M19" t="n">
-        <v>2.18</v>
+        <v>2.1867</v>
       </c>
       <c r="N19" t="inlineStr">
         <is>
@@ -1935,7 +1935,7 @@
         <v>25392</v>
       </c>
       <c r="F20" t="n">
-        <v>9.039999999999999</v>
+        <v>9.0382</v>
       </c>
       <c r="G20" t="n">
         <v>5976</v>
@@ -1956,7 +1956,7 @@
         <v>255549</v>
       </c>
       <c r="M20" t="n">
-        <v>0.23</v>
+        <v>0.2312</v>
       </c>
       <c r="N20" t="inlineStr">
         <is>
@@ -1998,7 +1998,7 @@
         <v>17230</v>
       </c>
       <c r="F21" t="n">
-        <v>7.32</v>
+        <v>7.3191</v>
       </c>
       <c r="G21" t="n">
         <v>6892</v>
@@ -2019,7 +2019,7 @@
         <v>218181</v>
       </c>
       <c r="M21" t="n">
-        <v>-3.51</v>
+        <v>-3.5134</v>
       </c>
       <c r="N21" t="inlineStr">
         <is>
@@ -2061,7 +2061,7 @@
         <v>22379</v>
       </c>
       <c r="F22" t="n">
-        <v>9.32</v>
+        <v>9.3187</v>
       </c>
       <c r="G22" t="n">
         <v>7533</v>
@@ -2082,7 +2082,7 @@
         <v>217773</v>
       </c>
       <c r="M22" t="n">
-        <v>-1.51</v>
+        <v>-1.5138</v>
       </c>
       <c r="N22" t="inlineStr">
         <is>
@@ -2124,7 +2124,7 @@
         <v>26496</v>
       </c>
       <c r="F23" t="n">
-        <v>11.14</v>
+        <v>11.144</v>
       </c>
       <c r="G23" t="n">
         <v>7570</v>
@@ -2145,7 +2145,7 @@
         <v>211264</v>
       </c>
       <c r="M23" t="n">
-        <v>0.31</v>
+        <v>0.3115</v>
       </c>
       <c r="N23" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         <v>26387</v>
       </c>
       <c r="F24" t="n">
-        <v>9.83</v>
+        <v>9.827199999999999</v>
       </c>
       <c r="G24" t="n">
         <v>8576</v>
@@ -2208,7 +2208,7 @@
         <v>242124</v>
       </c>
       <c r="M24" t="n">
-        <v>-1</v>
+        <v>-1.0053</v>
       </c>
       <c r="N24" t="inlineStr">
         <is>
@@ -2250,7 +2250,7 @@
         <v>33574</v>
       </c>
       <c r="F25" t="n">
-        <v>11.56</v>
+        <v>11.5595</v>
       </c>
       <c r="G25" t="n">
         <v>9259</v>
@@ -2271,7 +2271,7 @@
         <v>256871</v>
       </c>
       <c r="M25" t="n">
-        <v>0.73</v>
+        <v>0.727</v>
       </c>
       <c r="N25" t="inlineStr">
         <is>
@@ -2313,7 +2313,7 @@
         <v>45221</v>
       </c>
       <c r="F26" t="n">
-        <v>15.55</v>
+        <v>15.5455</v>
       </c>
       <c r="G26" t="n">
         <v>9658</v>
@@ -2334,7 +2334,7 @@
         <v>245673</v>
       </c>
       <c r="M26" t="n">
-        <v>4.72</v>
+        <v>4.713</v>
       </c>
       <c r="N26" t="inlineStr">
         <is>
@@ -2376,7 +2376,7 @@
         <v>22822</v>
       </c>
       <c r="F27" t="n">
-        <v>9.98</v>
+        <v>9.977600000000001</v>
       </c>
       <c r="G27" t="n">
         <v>6991</v>
@@ -2397,7 +2397,7 @@
         <v>205910</v>
       </c>
       <c r="M27" t="n">
-        <v>-0.85</v>
+        <v>-0.8549</v>
       </c>
       <c r="N27" t="inlineStr">
         <is>
@@ -2439,7 +2439,7 @@
         <v>29691</v>
       </c>
       <c r="F28" t="n">
-        <v>10.09</v>
+        <v>10.0925</v>
       </c>
       <c r="G28" t="n">
         <v>7369</v>
@@ -2460,7 +2460,7 @@
         <v>264499</v>
       </c>
       <c r="M28" t="n">
-        <v>1.49</v>
+        <v>1.4879</v>
       </c>
       <c r="N28" t="inlineStr">
         <is>
@@ -2502,7 +2502,7 @@
         <v>21963</v>
       </c>
       <c r="F29" t="n">
-        <v>7.38</v>
+        <v>7.3754</v>
       </c>
       <c r="G29" t="n">
         <v>7423</v>
@@ -2523,7 +2523,7 @@
         <v>275823</v>
       </c>
       <c r="M29" t="n">
-        <v>-1.22</v>
+        <v>-1.2292</v>
       </c>
       <c r="N29" t="inlineStr">
         <is>
@@ -2565,7 +2565,7 @@
         <v>27238</v>
       </c>
       <c r="F30" t="n">
-        <v>9.08</v>
+        <v>9.0778</v>
       </c>
       <c r="G30" t="n">
         <v>10155</v>
@@ -2586,7 +2586,7 @@
         <v>272813</v>
       </c>
       <c r="M30" t="n">
-        <v>0.48</v>
+        <v>0.4732</v>
       </c>
       <c r="N30" t="inlineStr">
         <is>
@@ -2628,7 +2628,7 @@
         <v>27593</v>
       </c>
       <c r="F31" t="n">
-        <v>8.42</v>
+        <v>8.424200000000001</v>
       </c>
       <c r="G31" t="n">
         <v>10031</v>
@@ -2649,7 +2649,7 @@
         <v>299951</v>
       </c>
       <c r="M31" t="n">
-        <v>-0.05</v>
+        <v>-0.0458</v>
       </c>
       <c r="N31" t="inlineStr">
         <is>
@@ -2691,7 +2691,7 @@
         <v>27236</v>
       </c>
       <c r="F32" t="n">
-        <v>9.710000000000001</v>
+        <v>9.7096</v>
       </c>
       <c r="G32" t="n">
         <v>10196</v>
@@ -2712,7 +2712,7 @@
         <v>253270</v>
       </c>
       <c r="M32" t="n">
-        <v>1.24</v>
+        <v>1.2396</v>
       </c>
       <c r="N32" t="inlineStr">
         <is>
@@ -2754,7 +2754,7 @@
         <v>17907</v>
       </c>
       <c r="F33" t="n">
-        <v>7.14</v>
+        <v>7.1427</v>
       </c>
       <c r="G33" t="n">
         <v>6906</v>
@@ -2775,7 +2775,7 @@
         <v>232796</v>
       </c>
       <c r="M33" t="n">
-        <v>-1.33</v>
+        <v>-1.3273</v>
       </c>
       <c r="N33" t="inlineStr">
         <is>
@@ -2817,7 +2817,7 @@
         <v>21018</v>
       </c>
       <c r="F34" t="n">
-        <v>7.81</v>
+        <v>7.8105</v>
       </c>
       <c r="G34" t="n">
         <v>8200</v>
@@ -2838,7 +2838,7 @@
         <v>248083</v>
       </c>
       <c r="M34" t="n">
-        <v>-0.79</v>
+        <v>-0.7941</v>
       </c>
       <c r="N34" t="inlineStr">
         <is>
@@ -2880,7 +2880,7 @@
         <v>25278</v>
       </c>
       <c r="F35" t="n">
-        <v>11</v>
+        <v>10.9981</v>
       </c>
       <c r="G35" t="n">
         <v>9362</v>
@@ -2901,7 +2901,7 @@
         <v>204561</v>
       </c>
       <c r="M35" t="n">
-        <v>-4.53</v>
+        <v>-4.5293</v>
       </c>
       <c r="N35" t="inlineStr">
         <is>
@@ -2943,7 +2943,7 @@
         <v>68540</v>
       </c>
       <c r="F36" t="n">
-        <v>16.82</v>
+        <v>16.8203</v>
       </c>
       <c r="G36" t="n">
         <v>15886</v>
@@ -2964,7 +2964,7 @@
         <v>338944</v>
       </c>
       <c r="M36" t="n">
-        <v>1.29</v>
+        <v>1.2929</v>
       </c>
       <c r="N36" t="inlineStr">
         <is>
@@ -3006,7 +3006,7 @@
         <v>51707</v>
       </c>
       <c r="F37" t="n">
-        <v>20.21</v>
+        <v>20.2062</v>
       </c>
       <c r="G37" t="n">
         <v>10596</v>
@@ -3027,7 +3027,7 @@
         <v>204190</v>
       </c>
       <c r="M37" t="n">
-        <v>4.68</v>
+        <v>4.6788</v>
       </c>
       <c r="N37" t="inlineStr">
         <is>
@@ -3069,7 +3069,7 @@
         <v>28186</v>
       </c>
       <c r="F38" t="n">
-        <v>11.65</v>
+        <v>11.6507</v>
       </c>
       <c r="G38" t="n">
         <v>11383</v>
@@ -3090,7 +3090,7 @@
         <v>213740</v>
       </c>
       <c r="M38" t="n">
-        <v>-3.88</v>
+        <v>-3.8767</v>
       </c>
       <c r="N38" t="inlineStr">
         <is>
@@ -3132,7 +3132,7 @@
         <v>42075</v>
       </c>
       <c r="F39" t="n">
-        <v>16.53</v>
+        <v>16.5281</v>
       </c>
       <c r="G39" t="n">
         <v>9449</v>
@@ -3153,7 +3153,7 @@
         <v>212491</v>
       </c>
       <c r="M39" t="n">
-        <v>1</v>
+        <v>1.0007</v>
       </c>
       <c r="N39" t="inlineStr">
         <is>
@@ -3195,7 +3195,7 @@
         <v>33831</v>
       </c>
       <c r="F40" t="n">
-        <v>10.91</v>
+        <v>10.9087</v>
       </c>
       <c r="G40" t="n">
         <v>11629</v>
@@ -3216,7 +3216,7 @@
         <v>276298</v>
       </c>
       <c r="M40" t="n">
-        <v>-12.3</v>
+        <v>-12.2988</v>
       </c>
       <c r="N40" t="inlineStr">
         <is>
@@ -3258,7 +3258,7 @@
         <v>35646</v>
       </c>
       <c r="F41" t="n">
-        <v>11.77</v>
+        <v>11.7684</v>
       </c>
       <c r="G41" t="n">
         <v>10998</v>
@@ -3279,7 +3279,7 @@
         <v>267250</v>
       </c>
       <c r="M41" t="n">
-        <v>-11.44</v>
+        <v>-11.4391</v>
       </c>
       <c r="N41" t="inlineStr">
         <is>
@@ -3321,7 +3321,7 @@
         <v>97085</v>
       </c>
       <c r="F42" t="n">
-        <v>21</v>
+        <v>21.0022</v>
       </c>
       <c r="G42" t="n">
         <v>12656</v>
@@ -3342,7 +3342,7 @@
         <v>365177</v>
       </c>
       <c r="M42" t="n">
-        <v>-2.21</v>
+        <v>-2.2053</v>
       </c>
       <c r="N42" t="inlineStr">
         <is>
@@ -3384,7 +3384,7 @@
         <v>107713</v>
       </c>
       <c r="F43" t="n">
-        <v>25.4</v>
+        <v>25.401</v>
       </c>
       <c r="G43" t="n">
         <v>18161</v>
@@ -3405,7 +3405,7 @@
         <v>316338</v>
       </c>
       <c r="M43" t="n">
-        <v>2.19</v>
+        <v>2.1935</v>
       </c>
       <c r="N43" t="inlineStr">
         <is>
@@ -3447,7 +3447,7 @@
         <v>114822</v>
       </c>
       <c r="F44" t="n">
-        <v>25.95</v>
+        <v>25.9529</v>
       </c>
       <c r="G44" t="n">
         <v>11627</v>
@@ -3468,7 +3468,7 @@
         <v>327603</v>
       </c>
       <c r="M44" t="n">
-        <v>2.74</v>
+        <v>2.7454</v>
       </c>
       <c r="N44" t="inlineStr">
         <is>
@@ -3510,7 +3510,7 @@
         <v>72317</v>
       </c>
       <c r="F45" t="n">
-        <v>27.16</v>
+        <v>27.1581</v>
       </c>
       <c r="G45" t="n">
         <v>15401</v>
@@ -3531,7 +3531,7 @@
         <v>193965</v>
       </c>
       <c r="M45" t="n">
-        <v>3.95</v>
+        <v>3.9506</v>
       </c>
       <c r="N45" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
         <v>74551</v>
       </c>
       <c r="F46" t="n">
-        <v>29.01</v>
+        <v>29.0059</v>
       </c>
       <c r="G46" t="n">
         <v>11759</v>
@@ -3594,7 +3594,7 @@
         <v>182469</v>
       </c>
       <c r="M46" t="n">
-        <v>5.8</v>
+        <v>5.7984</v>
       </c>
       <c r="N46" t="inlineStr">
         <is>
@@ -3636,7 +3636,7 @@
         <v>73338</v>
       </c>
       <c r="F47" t="n">
-        <v>27.38</v>
+        <v>27.376</v>
       </c>
       <c r="G47" t="n">
         <v>10361</v>
@@ -3657,7 +3657,7 @@
         <v>194554</v>
       </c>
       <c r="M47" t="n">
-        <v>4.17</v>
+        <v>4.1685</v>
       </c>
       <c r="N47" t="inlineStr">
         <is>
@@ -3699,7 +3699,7 @@
         <v>82407</v>
       </c>
       <c r="F48" t="n">
-        <v>26.86</v>
+        <v>26.8581</v>
       </c>
       <c r="G48" t="n">
         <v>13910</v>
@@ -3720,7 +3720,7 @@
         <v>224417</v>
       </c>
       <c r="M48" t="n">
-        <v>3.65</v>
+        <v>3.6506</v>
       </c>
       <c r="N48" t="inlineStr">
         <is>
@@ -3762,7 +3762,7 @@
         <v>69148</v>
       </c>
       <c r="F49" t="n">
-        <v>28.4</v>
+        <v>28.3974</v>
       </c>
       <c r="G49" t="n">
         <v>8075</v>
@@ -3783,7 +3783,7 @@
         <v>174353</v>
       </c>
       <c r="M49" t="n">
-        <v>5.19</v>
+        <v>5.1899</v>
       </c>
       <c r="N49" t="inlineStr">
         <is>
@@ -3825,7 +3825,7 @@
         <v>66511</v>
       </c>
       <c r="F50" t="n">
-        <v>30.71</v>
+        <v>30.7057</v>
       </c>
       <c r="G50" t="n">
         <v>11110</v>
@@ -3846,7 +3846,7 @@
         <v>150097</v>
       </c>
       <c r="M50" t="n">
-        <v>7.5</v>
+        <v>7.4982</v>
       </c>
       <c r="N50" t="inlineStr">
         <is>
@@ -3888,7 +3888,7 @@
         <v>88029</v>
       </c>
       <c r="F51" t="n">
-        <v>29.98</v>
+        <v>29.9777</v>
       </c>
       <c r="G51" t="n">
         <v>12090</v>
@@ -3909,7 +3909,7 @@
         <v>205619</v>
       </c>
       <c r="M51" t="n">
-        <v>6.77</v>
+        <v>6.7702</v>
       </c>
       <c r="N51" t="inlineStr">
         <is>
@@ -3951,7 +3951,7 @@
         <v>52385</v>
       </c>
       <c r="F52" t="n">
-        <v>25</v>
+        <v>24.9999</v>
       </c>
       <c r="G52" t="n">
         <v>12913</v>
@@ -3972,7 +3972,7 @@
         <v>157156</v>
       </c>
       <c r="M52" t="n">
-        <v>1.79</v>
+        <v>1.7924</v>
       </c>
       <c r="N52" t="inlineStr">
         <is>
@@ -4014,7 +4014,7 @@
         <v>51369</v>
       </c>
       <c r="F53" t="n">
-        <v>23.8</v>
+        <v>23.7981</v>
       </c>
       <c r="G53" t="n">
         <v>10565</v>
@@ -4035,7 +4035,7 @@
         <v>164484</v>
       </c>
       <c r="M53" t="n">
-        <v>0.59</v>
+        <v>0.5906</v>
       </c>
       <c r="N53" t="inlineStr">
         <is>
@@ -4077,7 +4077,7 @@
         <v>73989</v>
       </c>
       <c r="F54" t="n">
-        <v>26.57</v>
+        <v>26.5717</v>
       </c>
       <c r="G54" t="n">
         <v>11291</v>
@@ -4098,7 +4098,7 @@
         <v>204461</v>
       </c>
       <c r="M54" t="n">
-        <v>3.36</v>
+        <v>3.3642</v>
       </c>
       <c r="N54" t="inlineStr">
         <is>
@@ -4140,7 +4140,7 @@
         <v>69525</v>
       </c>
       <c r="F55" t="n">
-        <v>24.57</v>
+        <v>24.5743</v>
       </c>
       <c r="G55" t="n">
         <v>14029</v>
@@ -4161,7 +4161,7 @@
         <v>213392</v>
       </c>
       <c r="M55" t="n">
-        <v>1.36</v>
+        <v>1.3668</v>
       </c>
       <c r="N55" t="inlineStr">
         <is>
@@ -4203,7 +4203,7 @@
         <v>79834</v>
       </c>
       <c r="F56" t="n">
-        <v>27.72</v>
+        <v>27.7238</v>
       </c>
       <c r="G56" t="n">
         <v>10306</v>
@@ -4224,7 +4224,7 @@
         <v>208128</v>
       </c>
       <c r="M56" t="n">
-        <v>4.51</v>
+        <v>4.5163</v>
       </c>
       <c r="N56" t="inlineStr">
         <is>
@@ -4266,7 +4266,7 @@
         <v>59715</v>
       </c>
       <c r="F57" t="n">
-        <v>27.79</v>
+        <v>27.7937</v>
       </c>
       <c r="G57" t="n">
         <v>12383</v>
@@ -4287,7 +4287,7 @@
         <v>155136</v>
       </c>
       <c r="M57" t="n">
-        <v>4.58</v>
+        <v>4.5862</v>
       </c>
       <c r="N57" t="inlineStr">
         <is>
@@ -4329,7 +4329,7 @@
         <v>82579</v>
       </c>
       <c r="F58" t="n">
-        <v>19.11</v>
+        <v>19.1109</v>
       </c>
       <c r="G58" t="n">
         <v>15178</v>
@@ -4350,7 +4350,7 @@
         <v>349525</v>
       </c>
       <c r="M58" t="n">
-        <v>-4.1</v>
+        <v>-4.0966</v>
       </c>
       <c r="N58" t="inlineStr">
         <is>
@@ -4392,7 +4392,7 @@
         <v>29951</v>
       </c>
       <c r="F59" t="n">
-        <v>11.51</v>
+        <v>11.5148</v>
       </c>
       <c r="G59" t="n">
         <v>9522</v>
@@ -4413,7 +4413,7 @@
         <v>230157</v>
       </c>
       <c r="M59" t="n">
-        <v>-11.7</v>
+        <v>-11.6927</v>
       </c>
       <c r="N59" t="inlineStr">
         <is>
@@ -4455,7 +4455,7 @@
         <v>37959</v>
       </c>
       <c r="F60" t="n">
-        <v>13.35</v>
+        <v>13.3519</v>
       </c>
       <c r="G60" t="n">
         <v>9847</v>
@@ -4476,7 +4476,7 @@
         <v>246337</v>
       </c>
       <c r="M60" t="n">
-        <v>-9.859999999999999</v>
+        <v>-9.855600000000001</v>
       </c>
       <c r="N60" t="inlineStr">
         <is>
@@ -4518,7 +4518,7 @@
         <v>22584</v>
       </c>
       <c r="F61" t="n">
-        <v>8.25</v>
+        <v>8.2498</v>
       </c>
       <c r="G61" t="n">
         <v>6369</v>
@@ -4539,7 +4539,7 @@
         <v>251167</v>
       </c>
       <c r="M61" t="n">
-        <v>-1</v>
+        <v>-0.9967</v>
       </c>
       <c r="N61" t="inlineStr">
         <is>
@@ -4581,7 +4581,7 @@
         <v>23503</v>
       </c>
       <c r="F62" t="n">
-        <v>7.87</v>
+        <v>7.8734</v>
       </c>
       <c r="G62" t="n">
         <v>6956</v>
@@ -4602,7 +4602,7 @@
         <v>275008</v>
       </c>
       <c r="M62" t="n">
-        <v>-1.38</v>
+        <v>-1.3731</v>
       </c>
       <c r="N62" t="inlineStr">
         <is>
@@ -4644,7 +4644,7 @@
         <v>42795</v>
       </c>
       <c r="F63" t="n">
-        <v>13.68</v>
+        <v>13.6844</v>
       </c>
       <c r="G63" t="n">
         <v>14234</v>
@@ -4665,7 +4665,7 @@
         <v>269934</v>
       </c>
       <c r="M63" t="n">
-        <v>4.43</v>
+        <v>4.4379</v>
       </c>
       <c r="N63" t="inlineStr">
         <is>
@@ -4707,7 +4707,7 @@
         <v>22503</v>
       </c>
       <c r="F64" t="n">
-        <v>8.18</v>
+        <v>8.1807</v>
       </c>
       <c r="G64" t="n">
         <v>7123</v>
@@ -4728,7 +4728,7 @@
         <v>252570</v>
       </c>
       <c r="M64" t="n">
-        <v>-1.07</v>
+        <v>-1.0658</v>
       </c>
       <c r="N64" t="inlineStr">
         <is>
@@ -4770,7 +4770,7 @@
         <v>25647</v>
       </c>
       <c r="F65" t="n">
-        <v>7.97</v>
+        <v>7.9667</v>
       </c>
       <c r="G65" t="n">
         <v>8412</v>
@@ -4791,7 +4791,7 @@
         <v>296280</v>
       </c>
       <c r="M65" t="n">
-        <v>-1.28</v>
+        <v>-1.2798</v>
       </c>
       <c r="N65" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
         <v>28840</v>
       </c>
       <c r="F66" t="n">
-        <v>9.710000000000001</v>
+        <v>9.713200000000001</v>
       </c>
       <c r="G66" t="n">
         <v>10461</v>
@@ -4854,7 +4854,7 @@
         <v>268076</v>
       </c>
       <c r="M66" t="n">
-        <v>1.68</v>
+        <v>1.6818</v>
       </c>
       <c r="N66" t="inlineStr">
         <is>
@@ -4896,7 +4896,7 @@
         <v>13559</v>
       </c>
       <c r="F67" t="n">
-        <v>5.26</v>
+        <v>5.2633</v>
       </c>
       <c r="G67" t="n">
         <v>4682</v>
@@ -4917,7 +4917,7 @@
         <v>244055</v>
       </c>
       <c r="M67" t="n">
-        <v>-2.77</v>
+        <v>-2.7681</v>
       </c>
       <c r="N67" t="inlineStr">
         <is>
@@ -4959,7 +4959,7 @@
         <v>25879</v>
       </c>
       <c r="F68" t="n">
-        <v>8.75</v>
+        <v>8.7544</v>
       </c>
       <c r="G68" t="n">
         <v>8212</v>
@@ -4980,7 +4980,7 @@
         <v>269733</v>
       </c>
       <c r="M68" t="n">
-        <v>0.72</v>
+        <v>0.723</v>
       </c>
       <c r="N68" t="inlineStr">
         <is>
@@ -5022,7 +5022,7 @@
         <v>63582</v>
       </c>
       <c r="F69" t="n">
-        <v>20.59</v>
+        <v>20.5906</v>
       </c>
       <c r="G69" t="n">
         <v>14850</v>
@@ -5043,7 +5043,7 @@
         <v>245209</v>
       </c>
       <c r="M69" t="n">
-        <v>6.55</v>
+        <v>6.5519</v>
       </c>
       <c r="N69" t="inlineStr">
         <is>
@@ -5085,7 +5085,7 @@
         <v>73781</v>
       </c>
       <c r="F70" t="n">
-        <v>20.18</v>
+        <v>20.178</v>
       </c>
       <c r="G70" t="n">
         <v>15978</v>
@@ -5106,7 +5106,7 @@
         <v>291870</v>
       </c>
       <c r="M70" t="n">
-        <v>6.14</v>
+        <v>6.1393</v>
       </c>
       <c r="N70" t="inlineStr">
         <is>
@@ -5148,7 +5148,7 @@
         <v>53959</v>
       </c>
       <c r="F71" t="n">
-        <v>20.77</v>
+        <v>20.7651</v>
       </c>
       <c r="G71" t="n">
         <v>12337</v>
@@ -5169,7 +5169,7 @@
         <v>205895</v>
       </c>
       <c r="M71" t="n">
-        <v>6.73</v>
+        <v>6.7264</v>
       </c>
       <c r="N71" t="inlineStr">
         <is>
@@ -5211,7 +5211,7 @@
         <v>50371</v>
       </c>
       <c r="F72" t="n">
-        <v>12.6</v>
+        <v>12.5975</v>
       </c>
       <c r="G72" t="n">
         <v>10377</v>
@@ -5232,7 +5232,7 @@
         <v>349479</v>
       </c>
       <c r="M72" t="n">
-        <v>-1.44</v>
+        <v>-1.4412</v>
       </c>
       <c r="N72" t="inlineStr">
         <is>
@@ -5274,7 +5274,7 @@
         <v>13407</v>
       </c>
       <c r="F73" t="n">
-        <v>4.99</v>
+        <v>4.9927</v>
       </c>
       <c r="G73" t="n">
         <v>5572</v>
@@ -5295,7 +5295,7 @@
         <v>255124</v>
       </c>
       <c r="M73" t="n">
-        <v>-9.050000000000001</v>
+        <v>-9.045999999999999</v>
       </c>
       <c r="N73" t="inlineStr">
         <is>
@@ -5337,7 +5337,7 @@
         <v>24380</v>
       </c>
       <c r="F74" t="n">
-        <v>10.34</v>
+        <v>10.3373</v>
       </c>
       <c r="G74" t="n">
         <v>7312</v>
@@ -5358,7 +5358,7 @@
         <v>211466</v>
       </c>
       <c r="M74" t="n">
-        <v>-3.7</v>
+        <v>-3.7014</v>
       </c>
       <c r="N74" t="inlineStr">
         <is>
@@ -5400,7 +5400,7 @@
         <v>29601</v>
       </c>
       <c r="F75" t="n">
-        <v>10.51</v>
+        <v>10.5142</v>
       </c>
       <c r="G75" t="n">
         <v>11875</v>
@@ -5421,7 +5421,7 @@
         <v>251933</v>
       </c>
       <c r="M75" t="n">
-        <v>-3.53</v>
+        <v>-3.5245</v>
       </c>
       <c r="N75" t="inlineStr">
         <is>
@@ -5463,7 +5463,7 @@
         <v>26589</v>
       </c>
       <c r="F76" t="n">
-        <v>9.81</v>
+        <v>9.8125</v>
       </c>
       <c r="G76" t="n">
         <v>11252</v>
@@ -5484,7 +5484,7 @@
         <v>244381</v>
       </c>
       <c r="M76" t="n">
-        <v>-4.23</v>
+        <v>-4.2262</v>
       </c>
       <c r="N76" t="inlineStr">
         <is>
@@ -5526,7 +5526,7 @@
         <v>24275</v>
       </c>
       <c r="F77" t="n">
-        <v>10.38</v>
+        <v>10.3839</v>
       </c>
       <c r="G77" t="n">
         <v>7353</v>
@@ -5547,7 +5547,7 @@
         <v>209501</v>
       </c>
       <c r="M77" t="n">
-        <v>-3.92</v>
+        <v>-3.9161</v>
       </c>
       <c r="N77" t="inlineStr">
         <is>
@@ -5589,7 +5589,7 @@
         <v>30556</v>
       </c>
       <c r="F78" t="n">
-        <v>11.64</v>
+        <v>11.6403</v>
       </c>
       <c r="G78" t="n">
         <v>7572</v>
@@ -5610,7 +5610,7 @@
         <v>231946</v>
       </c>
       <c r="M78" t="n">
-        <v>-2.66</v>
+        <v>-2.6597</v>
       </c>
       <c r="N78" t="inlineStr">
         <is>
@@ -5652,7 +5652,7 @@
         <v>53622</v>
       </c>
       <c r="F79" t="n">
-        <v>19.18</v>
+        <v>19.1836</v>
       </c>
       <c r="G79" t="n">
         <v>10617</v>
@@ -5673,7 +5673,7 @@
         <v>225898</v>
       </c>
       <c r="M79" t="n">
-        <v>4.88</v>
+        <v>4.8836</v>
       </c>
       <c r="N79" t="inlineStr">
         <is>
@@ -5715,7 +5715,7 @@
         <v>47484</v>
       </c>
       <c r="F80" t="n">
-        <v>20.33</v>
+        <v>20.3338</v>
       </c>
       <c r="G80" t="n">
         <v>10745</v>
@@ -5736,7 +5736,7 @@
         <v>186039</v>
       </c>
       <c r="M80" t="n">
-        <v>6.03</v>
+        <v>6.0338</v>
       </c>
       <c r="N80" t="inlineStr">
         <is>
@@ -5778,7 +5778,7 @@
         <v>21540</v>
       </c>
       <c r="F81" t="n">
-        <v>9.289999999999999</v>
+        <v>9.2935</v>
       </c>
       <c r="G81" t="n">
         <v>6825</v>
@@ -5799,7 +5799,7 @@
         <v>210236</v>
       </c>
       <c r="M81" t="n">
-        <v>-5.01</v>
+        <v>-5.0065</v>
       </c>
       <c r="N81" t="inlineStr">
         <is>
@@ -5841,7 +5841,7 @@
         <v>36405</v>
       </c>
       <c r="F82" t="n">
-        <v>11.6</v>
+        <v>11.6031</v>
       </c>
       <c r="G82" t="n">
         <v>11755</v>
@@ -5862,7 +5862,7 @@
         <v>277347</v>
       </c>
       <c r="M82" t="n">
-        <v>-0.91</v>
+        <v>-0.9112</v>
       </c>
       <c r="N82" t="inlineStr">
         <is>
@@ -5904,7 +5904,7 @@
         <v>40502</v>
       </c>
       <c r="F83" t="n">
-        <v>13.46</v>
+        <v>13.4647</v>
       </c>
       <c r="G83" t="n">
         <v>11921</v>
@@ -5925,7 +5925,7 @@
         <v>260300</v>
       </c>
       <c r="M83" t="n">
-        <v>0.95</v>
+        <v>0.9504</v>
       </c>
       <c r="N83" t="inlineStr">
         <is>
@@ -5967,7 +5967,7 @@
         <v>40966</v>
       </c>
       <c r="F84" t="n">
-        <v>15.19</v>
+        <v>15.1907</v>
       </c>
       <c r="G84" t="n">
         <v>10407</v>
@@ -5988,7 +5988,7 @@
         <v>228713</v>
       </c>
       <c r="M84" t="n">
-        <v>1.88</v>
+        <v>1.8771</v>
       </c>
       <c r="N84" t="inlineStr">
         <is>
@@ -6030,7 +6030,7 @@
         <v>25834</v>
       </c>
       <c r="F85" t="n">
-        <v>11.13</v>
+        <v>11.1323</v>
       </c>
       <c r="G85" t="n">
         <v>8349</v>
@@ -6051,7 +6051,7 @@
         <v>206230</v>
       </c>
       <c r="M85" t="n">
-        <v>-2.18</v>
+        <v>-2.1813</v>
       </c>
       <c r="N85" t="inlineStr">
         <is>
@@ -6093,7 +6093,7 @@
         <v>22628</v>
       </c>
       <c r="F86" t="n">
-        <v>9.050000000000001</v>
+        <v>9.0528</v>
       </c>
       <c r="G86" t="n">
         <v>8487</v>
@@ -6114,7 +6114,7 @@
         <v>227327</v>
       </c>
       <c r="M86" t="n">
-        <v>-2.56</v>
+        <v>-2.5556</v>
       </c>
       <c r="N86" t="inlineStr">
         <is>
@@ -6156,7 +6156,7 @@
         <v>49697</v>
       </c>
       <c r="F87" t="n">
-        <v>16.76</v>
+        <v>16.7574</v>
       </c>
       <c r="G87" t="n">
         <v>14047</v>
@@ -6177,7 +6177,7 @@
         <v>246870</v>
       </c>
       <c r="M87" t="n">
-        <v>5.15</v>
+        <v>5.149</v>
       </c>
       <c r="N87" t="inlineStr">
         <is>
@@ -6219,7 +6219,7 @@
         <v>29043</v>
       </c>
       <c r="F88" t="n">
-        <v>11.09</v>
+        <v>11.0935</v>
       </c>
       <c r="G88" t="n">
         <v>9417</v>
@@ -6240,7 +6240,7 @@
         <v>232760</v>
       </c>
       <c r="M88" t="n">
-        <v>-0.52</v>
+        <v>-0.5149</v>
       </c>
       <c r="N88" t="inlineStr">
         <is>
@@ -6282,7 +6282,7 @@
         <v>26221</v>
       </c>
       <c r="F89" t="n">
-        <v>10.41</v>
+        <v>10.4119</v>
       </c>
       <c r="G89" t="n">
         <v>9775</v>
@@ -6303,7 +6303,7 @@
         <v>225615</v>
       </c>
       <c r="M89" t="n">
-        <v>-1.2</v>
+        <v>-1.1965</v>
       </c>
       <c r="N89" t="inlineStr">
         <is>
@@ -6345,7 +6345,7 @@
         <v>23360</v>
       </c>
       <c r="F90" t="n">
-        <v>9.73</v>
+        <v>9.725899999999999</v>
       </c>
       <c r="G90" t="n">
         <v>11290</v>
@@ -6366,7 +6366,7 @@
         <v>216823</v>
       </c>
       <c r="M90" t="n">
-        <v>-1.88</v>
+        <v>-1.8825</v>
       </c>
       <c r="N90" t="inlineStr">
         <is>
@@ -6408,7 +6408,7 @@
         <v>22765</v>
       </c>
       <c r="F91" t="n">
-        <v>8.380000000000001</v>
+        <v>8.3782</v>
       </c>
       <c r="G91" t="n">
         <v>9074</v>
@@ -6429,7 +6429,7 @@
         <v>248952</v>
       </c>
       <c r="M91" t="n">
-        <v>0.42</v>
+        <v>0.4207</v>
       </c>
       <c r="N91" t="inlineStr">
         <is>
@@ -6471,7 +6471,7 @@
         <v>18485</v>
       </c>
       <c r="F92" t="n">
-        <v>7.83</v>
+        <v>7.8291</v>
       </c>
       <c r="G92" t="n">
         <v>5981</v>
@@ -6492,7 +6492,7 @@
         <v>217620</v>
       </c>
       <c r="M92" t="n">
-        <v>-0.13</v>
+        <v>-0.1284</v>
       </c>
       <c r="N92" t="inlineStr">
         <is>
@@ -6534,7 +6534,7 @@
         <v>14895</v>
       </c>
       <c r="F93" t="n">
-        <v>6.2</v>
+        <v>6.2034</v>
       </c>
       <c r="G93" t="n">
         <v>5879</v>
@@ -6555,7 +6555,7 @@
         <v>225214</v>
       </c>
       <c r="M93" t="n">
-        <v>-1.76</v>
+        <v>-1.7541</v>
       </c>
       <c r="N93" t="inlineStr">
         <is>
@@ -6597,7 +6597,7 @@
         <v>25323</v>
       </c>
       <c r="F94" t="n">
-        <v>9.18</v>
+        <v>9.1799</v>
       </c>
       <c r="G94" t="n">
         <v>8862</v>
@@ -6618,7 +6618,7 @@
         <v>250531</v>
       </c>
       <c r="M94" t="n">
-        <v>1.22</v>
+        <v>1.2224</v>
       </c>
       <c r="N94" t="inlineStr">
         <is>
@@ -6660,7 +6660,7 @@
         <v>19194</v>
       </c>
       <c r="F95" t="n">
-        <v>8.59</v>
+        <v>8.5907</v>
       </c>
       <c r="G95" t="n">
         <v>5174</v>
@@ -6681,7 +6681,7 @@
         <v>204233</v>
       </c>
       <c r="M95" t="n">
-        <v>-2.31</v>
+        <v>-2.3077</v>
       </c>
       <c r="N95" t="inlineStr">
         <is>
@@ -6723,7 +6723,7 @@
         <v>36215</v>
       </c>
       <c r="F96" t="n">
-        <v>12.81</v>
+        <v>12.8079</v>
       </c>
       <c r="G96" t="n">
         <v>8052</v>
@@ -6744,7 +6744,7 @@
         <v>246540</v>
       </c>
       <c r="M96" t="n">
-        <v>1.91</v>
+        <v>1.9095</v>
       </c>
       <c r="N96" t="inlineStr">
         <is>
@@ -6786,7 +6786,7 @@
         <v>19654</v>
       </c>
       <c r="F97" t="n">
-        <v>8.59</v>
+        <v>8.594799999999999</v>
       </c>
       <c r="G97" t="n">
         <v>5121</v>
@@ -6807,7 +6807,7 @@
         <v>209020</v>
       </c>
       <c r="M97" t="n">
-        <v>-2.31</v>
+        <v>-2.3036</v>
       </c>
       <c r="N97" t="inlineStr">
         <is>
@@ -6849,7 +6849,7 @@
         <v>33752</v>
       </c>
       <c r="F98" t="n">
-        <v>13.25</v>
+        <v>13.2453</v>
       </c>
       <c r="G98" t="n">
         <v>9027</v>
@@ -6870,7 +6870,7 @@
         <v>221070</v>
       </c>
       <c r="M98" t="n">
-        <v>2.35</v>
+        <v>2.3469</v>
       </c>
       <c r="N98" t="inlineStr">
         <is>
@@ -6912,7 +6912,7 @@
         <v>29744</v>
       </c>
       <c r="F99" t="n">
-        <v>10.56</v>
+        <v>10.5589</v>
       </c>
       <c r="G99" t="n">
         <v>7373</v>
@@ -6933,7 +6933,7 @@
         <v>251953</v>
       </c>
       <c r="M99" t="n">
-        <v>-0.34</v>
+        <v>-0.3395</v>
       </c>
       <c r="N99" t="inlineStr">
         <is>
@@ -6975,7 +6975,7 @@
         <v>22959</v>
       </c>
       <c r="F100" t="n">
-        <v>9.18</v>
+        <v>9.175599999999999</v>
       </c>
       <c r="G100" t="n">
         <v>7179</v>
@@ -6996,7 +6996,7 @@
         <v>227258</v>
       </c>
       <c r="M100" t="n">
-        <v>-3.08</v>
+        <v>-3.0881</v>
       </c>
       <c r="N100" t="inlineStr">
         <is>
@@ -7038,7 +7038,7 @@
         <v>27507</v>
       </c>
       <c r="F101" t="n">
-        <v>10.63</v>
+        <v>10.6299</v>
       </c>
       <c r="G101" t="n">
         <v>8697</v>
@@ -7059,7 +7059,7 @@
         <v>231263</v>
       </c>
       <c r="M101" t="n">
-        <v>-1.63</v>
+        <v>-1.6338</v>
       </c>
       <c r="N101" t="inlineStr">
         <is>
@@ -7101,7 +7101,7 @@
         <v>24513</v>
       </c>
       <c r="F102" t="n">
-        <v>10.71</v>
+        <v>10.7141</v>
       </c>
       <c r="G102" t="n">
         <v>5585</v>
@@ -7122,7 +7122,7 @@
         <v>204278</v>
       </c>
       <c r="M102" t="n">
-        <v>-1.55</v>
+        <v>-1.5496</v>
       </c>
       <c r="N102" t="inlineStr">
         <is>
@@ -7164,7 +7164,7 @@
         <v>25652</v>
       </c>
       <c r="F103" t="n">
-        <v>9.02</v>
+        <v>9.0212</v>
       </c>
       <c r="G103" t="n">
         <v>7408</v>
@@ -7185,7 +7185,7 @@
         <v>258699</v>
       </c>
       <c r="M103" t="n">
-        <v>-3.24</v>
+        <v>-3.2425</v>
       </c>
       <c r="N103" t="inlineStr">
         <is>
@@ -7227,7 +7227,7 @@
         <v>27052</v>
       </c>
       <c r="F104" t="n">
-        <v>8.890000000000001</v>
+        <v>8.890499999999999</v>
       </c>
       <c r="G104" t="n">
         <v>9794</v>
@@ -7248,7 +7248,7 @@
         <v>277228</v>
       </c>
       <c r="M104" t="n">
-        <v>-3.37</v>
+        <v>-3.3732</v>
       </c>
       <c r="N104" t="inlineStr">
         <is>
@@ -7290,7 +7290,7 @@
         <v>47478</v>
       </c>
       <c r="F105" t="n">
-        <v>17.57</v>
+        <v>17.5685</v>
       </c>
       <c r="G105" t="n">
         <v>14912</v>
@@ -7311,7 +7311,7 @@
         <v>222767</v>
       </c>
       <c r="M105" t="n">
-        <v>5.31</v>
+        <v>5.3048</v>
       </c>
       <c r="N105" t="inlineStr">
         <is>
@@ -7353,7 +7353,7 @@
         <v>53795</v>
       </c>
       <c r="F106" t="n">
-        <v>19.9</v>
+        <v>19.9032</v>
       </c>
       <c r="G106" t="n">
         <v>12511</v>
@@ -7374,7 +7374,7 @@
         <v>216488</v>
       </c>
       <c r="M106" t="n">
-        <v>7.64</v>
+        <v>7.6395</v>
       </c>
       <c r="N106" t="inlineStr">
         <is>
@@ -7416,7 +7416,7 @@
         <v>22690</v>
       </c>
       <c r="F107" t="n">
-        <v>8.529999999999999</v>
+        <v>8.526999999999999</v>
       </c>
       <c r="G107" t="n">
         <v>6175</v>
@@ -7437,7 +7437,7 @@
         <v>243405</v>
       </c>
       <c r="M107" t="n">
-        <v>-0.48</v>
+        <v>-0.4803</v>
       </c>
       <c r="N107" t="inlineStr">
         <is>
@@ -7479,7 +7479,7 @@
         <v>27977</v>
       </c>
       <c r="F108" t="n">
-        <v>9.44</v>
+        <v>9.438499999999999</v>
       </c>
       <c r="G108" t="n">
         <v>6681</v>
@@ -7500,7 +7500,7 @@
         <v>268436</v>
       </c>
       <c r="M108" t="n">
-        <v>0.43</v>
+        <v>0.4312</v>
       </c>
       <c r="N108" t="inlineStr">
         <is>
@@ -7542,7 +7542,7 @@
         <v>22007</v>
       </c>
       <c r="F109" t="n">
-        <v>9.24</v>
+        <v>9.2399</v>
       </c>
       <c r="G109" t="n">
         <v>8710</v>
@@ -7563,7 +7563,7 @@
         <v>216166</v>
       </c>
       <c r="M109" t="n">
-        <v>-3.55</v>
+        <v>-3.5492</v>
       </c>
       <c r="N109" t="inlineStr">
         <is>
@@ -7605,7 +7605,7 @@
         <v>32538</v>
       </c>
       <c r="F110" t="n">
-        <v>12.15</v>
+        <v>12.1483</v>
       </c>
       <c r="G110" t="n">
         <v>11721</v>
@@ -7626,7 +7626,7 @@
         <v>235302</v>
       </c>
       <c r="M110" t="n">
-        <v>-0.64</v>
+        <v>-0.6408</v>
       </c>
       <c r="N110" t="inlineStr">
         <is>
@@ -7668,7 +7668,7 @@
         <v>25124</v>
       </c>
       <c r="F111" t="n">
-        <v>10.88</v>
+        <v>10.8756</v>
       </c>
       <c r="G111" t="n">
         <v>9995</v>
@@ -7689,7 +7689,7 @@
         <v>205889</v>
       </c>
       <c r="M111" t="n">
-        <v>-1.91</v>
+        <v>-1.9135</v>
       </c>
       <c r="N111" t="inlineStr">
         <is>
@@ -7731,7 +7731,7 @@
         <v>33659</v>
       </c>
       <c r="F112" t="n">
-        <v>12.11</v>
+        <v>12.1144</v>
       </c>
       <c r="G112" t="n">
         <v>12015</v>
@@ -7752,7 +7752,7 @@
         <v>244184</v>
       </c>
       <c r="M112" t="n">
-        <v>-0.68</v>
+        <v>-0.6747</v>
       </c>
       <c r="N112" t="inlineStr">
         <is>
@@ -7794,7 +7794,7 @@
         <v>74175</v>
       </c>
       <c r="F113" t="n">
-        <v>22.55</v>
+        <v>22.555</v>
       </c>
       <c r="G113" t="n">
         <v>11482</v>
@@ -7815,7 +7815,7 @@
         <v>254688</v>
       </c>
       <c r="M113" t="n">
-        <v>9.76</v>
+        <v>9.7659</v>
       </c>
       <c r="N113" t="inlineStr">
         <is>
@@ -7857,7 +7857,7 @@
         <v>24440</v>
       </c>
       <c r="F114" t="n">
-        <v>10.03</v>
+        <v>10.0305</v>
       </c>
       <c r="G114" t="n">
         <v>9027</v>
@@ -7878,7 +7878,7 @@
         <v>219217</v>
       </c>
       <c r="M114" t="n">
-        <v>-2.76</v>
+        <v>-2.7586</v>
       </c>
       <c r="N114" t="inlineStr">
         <is>
@@ -7920,7 +7920,7 @@
         <v>19837</v>
       </c>
       <c r="F115" t="n">
-        <v>8.82</v>
+        <v>8.818899999999999</v>
       </c>
       <c r="G115" t="n">
         <v>7304</v>
@@ -7941,7 +7941,7 @@
         <v>205101</v>
       </c>
       <c r="M115" t="n">
-        <v>-3.97</v>
+        <v>-3.9702</v>
       </c>
       <c r="N115" t="inlineStr">
         <is>
@@ -7983,7 +7983,7 @@
         <v>25474</v>
       </c>
       <c r="F116" t="n">
-        <v>9.83</v>
+        <v>9.833299999999999</v>
       </c>
       <c r="G116" t="n">
         <v>10519</v>
@@ -8004,7 +8004,7 @@
         <v>233585</v>
       </c>
       <c r="M116" t="n">
-        <v>-1.81</v>
+        <v>-1.8099</v>
       </c>
       <c r="N116" t="inlineStr">
         <is>
@@ -8046,7 +8046,7 @@
         <v>60119</v>
       </c>
       <c r="F117" t="n">
-        <v>21.35</v>
+        <v>21.346</v>
       </c>
       <c r="G117" t="n">
         <v>17143</v>
@@ -8067,7 +8067,7 @@
         <v>221521</v>
       </c>
       <c r="M117" t="n">
-        <v>9.710000000000001</v>
+        <v>9.7028</v>
       </c>
       <c r="N117" t="inlineStr">
         <is>
@@ -8109,7 +8109,7 @@
         <v>24580</v>
       </c>
       <c r="F118" t="n">
-        <v>9.43</v>
+        <v>9.433299999999999</v>
       </c>
       <c r="G118" t="n">
         <v>10785</v>
@@ -8130,7 +8130,7 @@
         <v>235987</v>
       </c>
       <c r="M118" t="n">
-        <v>-2.21</v>
+        <v>-2.2099</v>
       </c>
       <c r="N118" t="inlineStr">
         <is>
@@ -8172,7 +8172,7 @@
         <v>30389</v>
       </c>
       <c r="F119" t="n">
-        <v>11.55</v>
+        <v>11.5472</v>
       </c>
       <c r="G119" t="n">
         <v>13375</v>
@@ -8193,7 +8193,7 @@
         <v>232782</v>
       </c>
       <c r="M119" t="n">
-        <v>-0.09</v>
+        <v>-0.096</v>
       </c>
       <c r="N119" t="inlineStr">
         <is>
@@ -8235,7 +8235,7 @@
         <v>27735</v>
       </c>
       <c r="F120" t="n">
-        <v>9.91</v>
+        <v>9.909599999999999</v>
       </c>
       <c r="G120" t="n">
         <v>11695</v>
@@ -8256,7 +8256,7 @@
         <v>252144</v>
       </c>
       <c r="M120" t="n">
-        <v>-1.73</v>
+        <v>-1.7336</v>
       </c>
       <c r="N120" t="inlineStr">
         <is>
@@ -8298,7 +8298,7 @@
         <v>24405</v>
       </c>
       <c r="F121" t="n">
-        <v>7.85</v>
+        <v>7.8537</v>
       </c>
       <c r="G121" t="n">
         <v>9755</v>
@@ -8319,7 +8319,7 @@
         <v>286341</v>
       </c>
       <c r="M121" t="n">
-        <v>-3.79</v>
+        <v>-3.7895</v>
       </c>
       <c r="N121" t="inlineStr">
         <is>
@@ -8361,7 +8361,7 @@
         <v>24931</v>
       </c>
       <c r="F122" t="n">
-        <v>8.32</v>
+        <v>8.321999999999999</v>
       </c>
       <c r="G122" t="n">
         <v>11567</v>
@@ -8382,7 +8382,7 @@
         <v>274649</v>
       </c>
       <c r="M122" t="n">
-        <v>-0.13</v>
+        <v>-0.1242</v>
       </c>
       <c r="N122" t="inlineStr">
         <is>
@@ -8424,7 +8424,7 @@
         <v>22862</v>
       </c>
       <c r="F123" t="n">
-        <v>7.66</v>
+        <v>7.6627</v>
       </c>
       <c r="G123" t="n">
         <v>8946</v>
@@ -8445,7 +8445,7 @@
         <v>275494</v>
       </c>
       <c r="M123" t="n">
-        <v>-0.79</v>
+        <v>-0.7835</v>
       </c>
       <c r="N123" t="inlineStr">
         <is>
@@ -8487,7 +8487,7 @@
         <v>23954</v>
       </c>
       <c r="F124" t="n">
-        <v>9.52</v>
+        <v>9.5237</v>
       </c>
       <c r="G124" t="n">
         <v>8555</v>
@@ -8508,7 +8508,7 @@
         <v>227566</v>
       </c>
       <c r="M124" t="n">
-        <v>1.07</v>
+        <v>1.0775</v>
       </c>
       <c r="N124" t="inlineStr">
         <is>
@@ -8550,7 +8550,7 @@
         <v>17507</v>
       </c>
       <c r="F125" t="n">
-        <v>6.47</v>
+        <v>6.4748</v>
       </c>
       <c r="G125" t="n">
         <v>8978</v>
@@ -8571,7 +8571,7 @@
         <v>252879</v>
       </c>
       <c r="M125" t="n">
-        <v>-2.65</v>
+        <v>-2.6441</v>
       </c>
       <c r="N125" t="inlineStr">
         <is>
@@ -8613,7 +8613,7 @@
         <v>16341</v>
       </c>
       <c r="F126" t="n">
-        <v>6.93</v>
+        <v>6.9303</v>
       </c>
       <c r="G126" t="n">
         <v>6668</v>
@@ -8634,7 +8634,7 @@
         <v>219448</v>
       </c>
       <c r="M126" t="n">
-        <v>-2.19</v>
+        <v>-2.1886</v>
       </c>
       <c r="N126" t="inlineStr">
         <is>
@@ -8676,7 +8676,7 @@
         <v>31992</v>
       </c>
       <c r="F127" t="n">
-        <v>10.99</v>
+        <v>10.9933</v>
       </c>
       <c r="G127" t="n">
         <v>11553</v>
@@ -8697,7 +8697,7 @@
         <v>259022</v>
       </c>
       <c r="M127" t="n">
-        <v>1.87</v>
+        <v>1.8744</v>
       </c>
       <c r="N127" t="inlineStr">
         <is>
@@ -8739,7 +8739,7 @@
         <v>23025</v>
       </c>
       <c r="F128" t="n">
-        <v>8.609999999999999</v>
+        <v>8.606</v>
       </c>
       <c r="G128" t="n">
         <v>9952</v>
@@ -8760,7 +8760,7 @@
         <v>244522</v>
       </c>
       <c r="M128" t="n">
-        <v>-0.51</v>
+        <v>-0.5129</v>
       </c>
       <c r="N128" t="inlineStr">
         <is>
@@ -8802,7 +8802,7 @@
         <v>34135</v>
       </c>
       <c r="F129" t="n">
-        <v>12.01</v>
+        <v>12.0147</v>
       </c>
       <c r="G129" t="n">
         <v>12948</v>
@@ -8823,7 +8823,7 @@
         <v>249976</v>
       </c>
       <c r="M129" t="n">
-        <v>2.89</v>
+        <v>2.8958</v>
       </c>
       <c r="N129" t="inlineStr">
         <is>
@@ -8865,7 +8865,7 @@
         <v>34899</v>
       </c>
       <c r="F130" t="n">
-        <v>12.65</v>
+        <v>12.6522</v>
       </c>
       <c r="G130" t="n">
         <v>12611</v>
@@ -8886,7 +8886,7 @@
         <v>240935</v>
       </c>
       <c r="M130" t="n">
-        <v>2</v>
+        <v>2.0063</v>
       </c>
       <c r="N130" t="inlineStr">
         <is>
@@ -8928,7 +8928,7 @@
         <v>33128</v>
       </c>
       <c r="F131" t="n">
-        <v>11.21</v>
+        <v>11.2079</v>
       </c>
       <c r="G131" t="n">
         <v>11794</v>
@@ -8949,7 +8949,7 @@
         <v>262450</v>
       </c>
       <c r="M131" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.5620000000000001</v>
       </c>
       <c r="N131" t="inlineStr">
         <is>
@@ -8991,7 +8991,7 @@
         <v>20123</v>
       </c>
       <c r="F132" t="n">
-        <v>8.4</v>
+        <v>8.404400000000001</v>
       </c>
       <c r="G132" t="n">
         <v>7567</v>
@@ -9012,7 +9012,7 @@
         <v>219310</v>
       </c>
       <c r="M132" t="n">
-        <v>-2.25</v>
+        <v>-2.2415</v>
       </c>
       <c r="N132" t="inlineStr">
         <is>
@@ -9054,7 +9054,7 @@
         <v>43402</v>
       </c>
       <c r="F133" t="n">
-        <v>14.8</v>
+        <v>14.8018</v>
       </c>
       <c r="G133" t="n">
         <v>8326</v>
@@ -9075,7 +9075,7 @@
         <v>249819</v>
       </c>
       <c r="M133" t="n">
-        <v>4.15</v>
+        <v>4.1559</v>
       </c>
       <c r="N133" t="inlineStr">
         <is>
@@ -9117,7 +9117,7 @@
         <v>28882</v>
       </c>
       <c r="F134" t="n">
-        <v>9.33</v>
+        <v>9.3264</v>
       </c>
       <c r="G134" t="n">
         <v>10130</v>
@@ -9138,7 +9138,7 @@
         <v>280798</v>
       </c>
       <c r="M134" t="n">
-        <v>-1.32</v>
+        <v>-1.3195</v>
       </c>
       <c r="N134" t="inlineStr">
         <is>
@@ -9180,7 +9180,7 @@
         <v>19801</v>
       </c>
       <c r="F135" t="n">
-        <v>7.09</v>
+        <v>7.0906</v>
       </c>
       <c r="G135" t="n">
         <v>8112</v>
@@ -9201,7 +9201,7 @@
         <v>259455</v>
       </c>
       <c r="M135" t="n">
-        <v>-3.56</v>
+        <v>-3.5553</v>
       </c>
       <c r="N135" t="inlineStr">
         <is>
@@ -9243,7 +9243,7 @@
         <v>27987</v>
       </c>
       <c r="F136" t="n">
-        <v>11.84</v>
+        <v>11.8369</v>
       </c>
       <c r="G136" t="n">
         <v>11331</v>
@@ -9264,7 +9264,7 @@
         <v>208451</v>
       </c>
       <c r="M136" t="n">
-        <v>-6.9</v>
+        <v>-6.902</v>
       </c>
       <c r="N136" t="inlineStr">
         <is>
@@ -9306,7 +9306,7 @@
         <v>35489</v>
       </c>
       <c r="F137" t="n">
-        <v>13.92</v>
+        <v>13.9215</v>
       </c>
       <c r="G137" t="n">
         <v>13735</v>
@@ -9327,7 +9327,7 @@
         <v>219434</v>
       </c>
       <c r="M137" t="n">
-        <v>-4.82</v>
+        <v>-4.8174</v>
       </c>
       <c r="N137" t="inlineStr">
         <is>
@@ -9369,7 +9369,7 @@
         <v>22768</v>
       </c>
       <c r="F138" t="n">
-        <v>8.01</v>
+        <v>8.005699999999999</v>
       </c>
       <c r="G138" t="n">
         <v>10128</v>
@@ -9390,7 +9390,7 @@
         <v>261631</v>
       </c>
       <c r="M138" t="n">
-        <v>0.25</v>
+        <v>0.2488</v>
       </c>
       <c r="N138" t="inlineStr">
         <is>
@@ -9432,7 +9432,7 @@
         <v>17960</v>
       </c>
       <c r="F139" t="n">
-        <v>6.49</v>
+        <v>6.4853</v>
       </c>
       <c r="G139" t="n">
         <v>8166</v>
@@ -9453,7 +9453,7 @@
         <v>258973</v>
       </c>
       <c r="M139" t="n">
-        <v>-1.27</v>
+        <v>-1.2716</v>
       </c>
       <c r="N139" t="inlineStr">
         <is>
@@ -9495,7 +9495,7 @@
         <v>24607</v>
       </c>
       <c r="F140" t="n">
-        <v>8.76</v>
+        <v>8.758599999999999</v>
       </c>
       <c r="G140" t="n">
         <v>9353</v>
@@ -9516,7 +9516,7 @@
         <v>256341</v>
       </c>
       <c r="M140" t="n">
-        <v>1</v>
+        <v>1.0017</v>
       </c>
       <c r="N140" t="inlineStr">
         <is>
@@ -9558,7 +9558,7 @@
         <v>31483</v>
       </c>
       <c r="F141" t="n">
-        <v>12.88</v>
+        <v>12.8811</v>
       </c>
       <c r="G141" t="n">
         <v>13640</v>
@@ -9579,7 +9579,7 @@
         <v>212929</v>
       </c>
       <c r="M141" t="n">
-        <v>-5.86</v>
+        <v>-5.8578</v>
       </c>
       <c r="N141" t="inlineStr">
         <is>
@@ -9621,7 +9621,7 @@
         <v>74799</v>
       </c>
       <c r="F142" t="n">
-        <v>23.27</v>
+        <v>23.2711</v>
       </c>
       <c r="G142" t="n">
         <v>19067</v>
@@ -9642,7 +9642,7 @@
         <v>246625</v>
       </c>
       <c r="M142" t="n">
-        <v>4.53</v>
+        <v>4.5322</v>
       </c>
       <c r="N142" t="inlineStr">
         <is>
@@ -9684,7 +9684,7 @@
         <v>71775</v>
       </c>
       <c r="F143" t="n">
-        <v>23.49</v>
+        <v>23.4947</v>
       </c>
       <c r="G143" t="n">
         <v>14783</v>
@@ -9705,7 +9705,7 @@
         <v>233719</v>
       </c>
       <c r="M143" t="n">
-        <v>4.75</v>
+        <v>4.7558</v>
       </c>
       <c r="N143" t="inlineStr">
         <is>
@@ -9747,7 +9747,7 @@
         <v>62799</v>
       </c>
       <c r="F144" t="n">
-        <v>22.15</v>
+        <v>22.1523</v>
       </c>
       <c r="G144" t="n">
         <v>14033</v>
@@ -9768,7 +9768,7 @@
         <v>220688</v>
       </c>
       <c r="M144" t="n">
-        <v>3.41</v>
+        <v>3.4134</v>
       </c>
       <c r="N144" t="inlineStr">
         <is>
@@ -9810,7 +9810,7 @@
         <v>82632</v>
       </c>
       <c r="F145" t="n">
-        <v>27</v>
+        <v>26.9995</v>
       </c>
       <c r="G145" t="n">
         <v>23551</v>
@@ -9831,7 +9831,7 @@
         <v>223418</v>
       </c>
       <c r="M145" t="n">
-        <v>8.26</v>
+        <v>8.2606</v>
       </c>
       <c r="N145" t="inlineStr">
         <is>
@@ -9873,7 +9873,7 @@
         <v>59933</v>
       </c>
       <c r="F146" t="n">
-        <v>22</v>
+        <v>22.0026</v>
       </c>
       <c r="G146" t="n">
         <v>12816</v>
@@ -9894,7 +9894,7 @@
         <v>212458</v>
       </c>
       <c r="M146" t="n">
-        <v>3.26</v>
+        <v>3.2637</v>
       </c>
       <c r="N146" t="inlineStr">
         <is>
@@ -9936,7 +9936,7 @@
         <v>29779</v>
       </c>
       <c r="F147" t="n">
-        <v>12.05</v>
+        <v>12.0548</v>
       </c>
       <c r="G147" t="n">
         <v>13307</v>
@@ -9957,7 +9957,7 @@
         <v>217252</v>
       </c>
       <c r="M147" t="n">
-        <v>-6.69</v>
+        <v>-6.6841</v>
       </c>
       <c r="N147" t="inlineStr">
         <is>
@@ -9999,7 +9999,7 @@
         <v>27236</v>
       </c>
       <c r="F148" t="n">
-        <v>12.52</v>
+        <v>12.5242</v>
       </c>
       <c r="G148" t="n">
         <v>10459</v>
@@ -10020,7 +10020,7 @@
         <v>190231</v>
       </c>
       <c r="M148" t="n">
-        <v>-6.22</v>
+        <v>-6.2147</v>
       </c>
       <c r="N148" t="inlineStr">
         <is>
@@ -10062,7 +10062,7 @@
         <v>21684</v>
       </c>
       <c r="F149" t="n">
-        <v>9.1</v>
+        <v>9.1008</v>
       </c>
       <c r="G149" t="n">
         <v>8436</v>
@@ -10083,7 +10083,7 @@
         <v>216581</v>
       </c>
       <c r="M149" t="n">
-        <v>1.66</v>
+        <v>1.6599</v>
       </c>
       <c r="N149" t="inlineStr">
         <is>
@@ -10125,7 +10125,7 @@
         <v>13250</v>
       </c>
       <c r="F150" t="n">
-        <v>5.73</v>
+        <v>5.7304</v>
       </c>
       <c r="G150" t="n">
         <v>5470</v>
@@ -10146,7 +10146,7 @@
         <v>217972</v>
       </c>
       <c r="M150" t="n">
-        <v>-1.71</v>
+        <v>-1.7105</v>
       </c>
       <c r="N150" t="inlineStr">
         <is>
@@ -10188,7 +10188,7 @@
         <v>30132</v>
       </c>
       <c r="F151" t="n">
-        <v>12.08</v>
+        <v>12.0784</v>
       </c>
       <c r="G151" t="n">
         <v>10392</v>
@@ -10251,7 +10251,7 @@
         <v>31204</v>
       </c>
       <c r="F152" t="n">
-        <v>13.65</v>
+        <v>13.6542</v>
       </c>
       <c r="G152" t="n">
         <v>14235</v>
@@ -10272,7 +10272,7 @@
         <v>197326</v>
       </c>
       <c r="M152" t="n">
-        <v>-2.77</v>
+        <v>-2.7642</v>
       </c>
       <c r="N152" t="inlineStr">
         <is>
@@ -10314,7 +10314,7 @@
         <v>29877</v>
       </c>
       <c r="F153" t="n">
-        <v>11.28</v>
+        <v>11.2757</v>
       </c>
       <c r="G153" t="n">
         <v>15865</v>
@@ -10335,7 +10335,7 @@
         <v>235092</v>
       </c>
       <c r="M153" t="n">
-        <v>-5.14</v>
+        <v>-5.1427</v>
       </c>
       <c r="N153" t="inlineStr">
         <is>
@@ -10377,7 +10377,7 @@
         <v>66593</v>
       </c>
       <c r="F154" t="n">
-        <v>21.82</v>
+        <v>21.8247</v>
       </c>
       <c r="G154" t="n">
         <v>16589</v>
@@ -10398,7 +10398,7 @@
         <v>238534</v>
       </c>
       <c r="M154" t="n">
-        <v>5.4</v>
+        <v>5.4063</v>
       </c>
       <c r="N154" t="inlineStr">
         <is>
@@ -10440,7 +10440,7 @@
         <v>57374</v>
       </c>
       <c r="F155" t="n">
-        <v>21.86</v>
+        <v>21.8565</v>
       </c>
       <c r="G155" t="n">
         <v>11026</v>
@@ -10461,7 +10461,7 @@
         <v>205129</v>
       </c>
       <c r="M155" t="n">
-        <v>5.44</v>
+        <v>5.4381</v>
       </c>
       <c r="N155" t="inlineStr">
         <is>
@@ -10503,7 +10503,7 @@
         <v>105232</v>
       </c>
       <c r="F156" t="n">
-        <v>22.19</v>
+        <v>22.195</v>
       </c>
       <c r="G156" t="n">
         <v>11886</v>
@@ -10524,7 +10524,7 @@
         <v>368893</v>
       </c>
       <c r="M156" t="n">
-        <v>-3.47</v>
+        <v>-3.4604</v>
       </c>
       <c r="N156" t="inlineStr">
         <is>
@@ -10566,7 +10566,7 @@
         <v>31224</v>
       </c>
       <c r="F157" t="n">
-        <v>13.39</v>
+        <v>13.3895</v>
       </c>
       <c r="G157" t="n">
         <v>11163</v>
@@ -10587,7 +10587,7 @@
         <v>201974</v>
       </c>
       <c r="M157" t="n">
-        <v>-12.27</v>
+        <v>-12.2659</v>
       </c>
       <c r="N157" t="inlineStr">
         <is>
@@ -10629,7 +10629,7 @@
         <v>21512</v>
       </c>
       <c r="F158" t="n">
-        <v>8.65</v>
+        <v>8.6509</v>
       </c>
       <c r="G158" t="n">
         <v>9986</v>
@@ -10650,7 +10650,7 @@
         <v>227155</v>
       </c>
       <c r="M158" t="n">
-        <v>-17.01</v>
+        <v>-17.0045</v>
       </c>
       <c r="N158" t="inlineStr">
         <is>
@@ -10692,7 +10692,7 @@
         <v>156733</v>
       </c>
       <c r="F159" t="n">
-        <v>27.37</v>
+        <v>27.3667</v>
       </c>
       <c r="G159" t="n">
         <v>13757</v>
@@ -10713,7 +10713,7 @@
         <v>415982</v>
       </c>
       <c r="M159" t="n">
-        <v>1.71</v>
+        <v>1.7113</v>
       </c>
       <c r="N159" t="inlineStr">
         <is>
@@ -10755,7 +10755,7 @@
         <v>47325</v>
       </c>
       <c r="F160" t="n">
-        <v>21.84</v>
+        <v>21.8395</v>
       </c>
       <c r="G160" t="n">
         <v>11142</v>
@@ -10776,7 +10776,7 @@
         <v>169370</v>
       </c>
       <c r="M160" t="n">
-        <v>-3.82</v>
+        <v>-3.8159</v>
       </c>
       <c r="N160" t="inlineStr">
         <is>
@@ -10818,7 +10818,7 @@
         <v>42306</v>
       </c>
       <c r="F161" t="n">
-        <v>26.61</v>
+        <v>26.6072</v>
       </c>
       <c r="G161" t="n">
         <v>6549</v>
@@ -10839,7 +10839,7 @@
         <v>116696</v>
       </c>
       <c r="M161" t="n">
-        <v>0.95</v>
+        <v>0.9518</v>
       </c>
       <c r="N161" t="inlineStr">
         <is>
@@ -10881,7 +10881,7 @@
         <v>71275</v>
       </c>
       <c r="F162" t="n">
-        <v>34.11</v>
+        <v>34.1127</v>
       </c>
       <c r="G162" t="n">
         <v>3423</v>
@@ -10902,7 +10902,7 @@
         <v>137665</v>
       </c>
       <c r="M162" t="n">
-        <v>8.449999999999999</v>
+        <v>8.4573</v>
       </c>
       <c r="N162" t="inlineStr">
         <is>
@@ -10944,7 +10944,7 @@
         <v>62446</v>
       </c>
       <c r="F163" t="n">
-        <v>38.44</v>
+        <v>38.4437</v>
       </c>
       <c r="G163" t="n">
         <v>2673</v>
@@ -10965,7 +10965,7 @@
         <v>99989</v>
       </c>
       <c r="M163" t="n">
-        <v>12.78</v>
+        <v>12.7883</v>
       </c>
       <c r="N163" t="inlineStr">
         <is>
@@ -11007,7 +11007,7 @@
         <v>105114</v>
       </c>
       <c r="F164" t="n">
-        <v>33.73</v>
+        <v>33.7346</v>
       </c>
       <c r="G164" t="n">
         <v>8082</v>
@@ -11028,7 +11028,7 @@
         <v>206477</v>
       </c>
       <c r="M164" t="n">
-        <v>8.07</v>
+        <v>8.0792</v>
       </c>
       <c r="N164" t="inlineStr">
         <is>
@@ -11070,7 +11070,7 @@
         <v>98857</v>
       </c>
       <c r="F165" t="n">
-        <v>36.6</v>
+        <v>36.598</v>
       </c>
       <c r="G165" t="n">
         <v>6696</v>
@@ -11091,7 +11091,7 @@
         <v>171259</v>
       </c>
       <c r="M165" t="n">
-        <v>10.94</v>
+        <v>10.9426</v>
       </c>
       <c r="N165" t="inlineStr">
         <is>
@@ -11133,7 +11133,7 @@
         <v>85669</v>
       </c>
       <c r="F166" t="n">
-        <v>30.13</v>
+        <v>30.1323</v>
       </c>
       <c r="G166" t="n">
         <v>8247</v>
@@ -11154,7 +11154,7 @@
         <v>198641</v>
       </c>
       <c r="M166" t="n">
-        <v>4.47</v>
+        <v>4.4769</v>
       </c>
       <c r="N166" t="inlineStr">
         <is>
@@ -11196,7 +11196,7 @@
         <v>84976</v>
       </c>
       <c r="F167" t="n">
-        <v>25.95</v>
+        <v>25.9489</v>
       </c>
       <c r="G167" t="n">
         <v>5667</v>
@@ -11217,7 +11217,7 @@
         <v>242499</v>
       </c>
       <c r="M167" t="n">
-        <v>0.29</v>
+        <v>0.2935</v>
       </c>
       <c r="N167" t="inlineStr">
         <is>
@@ -11259,7 +11259,7 @@
         <v>53927</v>
       </c>
       <c r="F168" t="n">
-        <v>20.33</v>
+        <v>20.3306</v>
       </c>
       <c r="G168" t="n">
         <v>9754</v>
@@ -11280,7 +11280,7 @@
         <v>211323</v>
       </c>
       <c r="M168" t="n">
-        <v>-5.33</v>
+        <v>-5.3248</v>
       </c>
       <c r="N168" t="inlineStr">
         <is>
@@ -11322,7 +11322,7 @@
         <v>194506</v>
       </c>
       <c r="F169" t="n">
-        <v>31.72</v>
+        <v>31.7162</v>
       </c>
       <c r="G169" t="n">
         <v>13126</v>
@@ -11343,7 +11343,7 @@
         <v>418764</v>
       </c>
       <c r="M169" t="n">
-        <v>6.06</v>
+        <v>6.0608</v>
       </c>
       <c r="N169" t="inlineStr">
         <is>
@@ -11385,7 +11385,7 @@
         <v>65329</v>
       </c>
       <c r="F170" t="n">
-        <v>22.25</v>
+        <v>22.2472</v>
       </c>
       <c r="G170" t="n">
         <v>12098</v>
@@ -11406,7 +11406,7 @@
         <v>228321</v>
       </c>
       <c r="M170" t="n">
-        <v>-3.41</v>
+        <v>-3.4082</v>
       </c>
       <c r="N170" t="inlineStr">
         <is>
@@ -11448,7 +11448,7 @@
         <v>23888</v>
       </c>
       <c r="F171" t="n">
-        <v>10.29</v>
+        <v>10.2933</v>
       </c>
       <c r="G171" t="n">
         <v>12884</v>
@@ -11469,7 +11469,7 @@
         <v>208185</v>
       </c>
       <c r="M171" t="n">
-        <v>-15.37</v>
+        <v>-15.3621</v>
       </c>
       <c r="N171" t="inlineStr">
         <is>
@@ -11511,7 +11511,7 @@
         <v>14901</v>
       </c>
       <c r="F172" t="n">
-        <v>6.66</v>
+        <v>6.6586</v>
       </c>
       <c r="G172" t="n">
         <v>6006</v>
@@ -11532,7 +11532,7 @@
         <v>208886</v>
       </c>
       <c r="M172" t="n">
-        <v>-1.28</v>
+        <v>-1.2821</v>
       </c>
       <c r="N172" t="inlineStr">
         <is>
@@ -11574,7 +11574,7 @@
         <v>26025</v>
       </c>
       <c r="F173" t="n">
-        <v>8.92</v>
+        <v>8.9246</v>
       </c>
       <c r="G173" t="n">
         <v>9911</v>
@@ -11595,7 +11595,7 @@
         <v>265584</v>
       </c>
       <c r="M173" t="n">
-        <v>0.98</v>
+        <v>0.9839</v>
       </c>
       <c r="N173" t="inlineStr">
         <is>
@@ -11637,7 +11637,7 @@
         <v>11121</v>
       </c>
       <c r="F174" t="n">
-        <v>5.51</v>
+        <v>5.5141</v>
       </c>
       <c r="G174" t="n">
         <v>3963</v>
@@ -11700,7 +11700,7 @@
         <v>41445</v>
       </c>
       <c r="F175" t="n">
-        <v>17.24</v>
+        <v>17.2369</v>
       </c>
       <c r="G175" t="n">
         <v>10140</v>
@@ -11721,7 +11721,7 @@
         <v>198999</v>
       </c>
       <c r="M175" t="n">
-        <v>4.78</v>
+        <v>4.7756</v>
       </c>
       <c r="N175" t="inlineStr">
         <is>
@@ -11763,7 +11763,7 @@
         <v>46506</v>
       </c>
       <c r="F176" t="n">
-        <v>18.23</v>
+        <v>18.2331</v>
       </c>
       <c r="G176" t="n">
         <v>12245</v>
@@ -11784,7 +11784,7 @@
         <v>208557</v>
       </c>
       <c r="M176" t="n">
-        <v>5.77</v>
+        <v>5.7718</v>
       </c>
       <c r="N176" t="inlineStr">
         <is>
@@ -11826,7 +11826,7 @@
         <v>30919</v>
       </c>
       <c r="F177" t="n">
-        <v>10.44</v>
+        <v>10.4369</v>
       </c>
       <c r="G177" t="n">
         <v>12743</v>
@@ -11847,7 +11847,7 @@
         <v>265329</v>
       </c>
       <c r="M177" t="n">
-        <v>-2.02</v>
+        <v>-2.0244</v>
       </c>
       <c r="N177" t="inlineStr">
         <is>
@@ -11889,7 +11889,7 @@
         <v>17693</v>
       </c>
       <c r="F178" t="n">
-        <v>5.82</v>
+        <v>5.8173</v>
       </c>
       <c r="G178" t="n">
         <v>9074</v>
@@ -11910,7 +11910,7 @@
         <v>286452</v>
       </c>
       <c r="M178" t="n">
-        <v>-6.64</v>
+        <v>-6.644</v>
       </c>
       <c r="N178" t="inlineStr">
         <is>
@@ -11952,7 +11952,7 @@
         <v>15524</v>
       </c>
       <c r="F179" t="n">
-        <v>6.02</v>
+        <v>6.0169</v>
       </c>
       <c r="G179" t="n">
         <v>6191</v>
@@ -11973,7 +11973,7 @@
         <v>242481</v>
       </c>
       <c r="M179" t="n">
-        <v>-10.32</v>
+        <v>-10.3235</v>
       </c>
       <c r="N179" t="inlineStr">
         <is>
@@ -12015,7 +12015,7 @@
         <v>39703</v>
       </c>
       <c r="F180" t="n">
-        <v>14.68</v>
+        <v>14.6841</v>
       </c>
       <c r="G180" t="n">
         <v>11309</v>
@@ -12036,7 +12036,7 @@
         <v>230677</v>
       </c>
       <c r="M180" t="n">
-        <v>-1.66</v>
+        <v>-1.6563</v>
       </c>
       <c r="N180" t="inlineStr">
         <is>
@@ -12078,7 +12078,7 @@
         <v>75368</v>
       </c>
       <c r="F181" t="n">
-        <v>27.02</v>
+        <v>27.0221</v>
       </c>
       <c r="G181" t="n">
         <v>8616</v>
@@ -12099,7 +12099,7 @@
         <v>203544</v>
       </c>
       <c r="M181" t="n">
-        <v>10.68</v>
+        <v>10.6817</v>
       </c>
       <c r="N181" t="inlineStr">
         <is>
@@ -12141,7 +12141,7 @@
         <v>26799</v>
       </c>
       <c r="F182" t="n">
-        <v>9.56</v>
+        <v>9.5581</v>
       </c>
       <c r="G182" t="n">
         <v>9770</v>
@@ -12162,7 +12162,7 @@
         <v>253582</v>
       </c>
       <c r="M182" t="n">
-        <v>-6.78</v>
+        <v>-6.7823</v>
       </c>
       <c r="N182" t="inlineStr">
         <is>
@@ -12204,7 +12204,7 @@
         <v>69003</v>
       </c>
       <c r="F183" t="n">
-        <v>23.17</v>
+        <v>23.1687</v>
       </c>
       <c r="G183" t="n">
         <v>11341</v>
@@ -12225,7 +12225,7 @@
         <v>228826</v>
       </c>
       <c r="M183" t="n">
-        <v>6.83</v>
+        <v>6.8283</v>
       </c>
       <c r="N183" t="inlineStr">
         <is>
@@ -12382,7 +12382,7 @@
         <v>214175</v>
       </c>
       <c r="E2" t="n">
-        <v>12.67</v>
+        <v>12.6687</v>
       </c>
       <c r="F2" t="n">
         <v>55374</v>
@@ -12418,7 +12418,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>11.52</v>
+        <v>11.5226</v>
       </c>
     </row>
     <row r="3">
@@ -12437,7 +12437,7 @@
         <v>219627</v>
       </c>
       <c r="E3" t="n">
-        <v>8.369999999999999</v>
+        <v>8.366899999999999</v>
       </c>
       <c r="F3" t="n">
         <v>65122</v>
@@ -12473,7 +12473,7 @@
         <v>1</v>
       </c>
       <c r="Q3" t="n">
-        <v>7.57</v>
+        <v>7.5721</v>
       </c>
     </row>
     <row r="4">
@@ -12492,7 +12492,7 @@
         <v>107366</v>
       </c>
       <c r="E4" t="n">
-        <v>8.81</v>
+        <v>8.807</v>
       </c>
       <c r="F4" t="n">
         <v>25432</v>
@@ -12528,7 +12528,7 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>8.17</v>
+        <v>8.168200000000001</v>
       </c>
     </row>
     <row r="5">
@@ -12547,7 +12547,7 @@
         <v>194109</v>
       </c>
       <c r="E5" t="n">
-        <v>10.83</v>
+        <v>10.8325</v>
       </c>
       <c r="F5" t="n">
         <v>56479</v>
@@ -12583,7 +12583,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>9.449999999999999</v>
+        <v>9.4518</v>
       </c>
     </row>
     <row r="6">
@@ -12602,7 +12602,7 @@
         <v>99910</v>
       </c>
       <c r="E6" t="n">
-        <v>8.6</v>
+        <v>8.6046</v>
       </c>
       <c r="F6" t="n">
         <v>33147</v>
@@ -12638,7 +12638,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>7.22</v>
+        <v>7.2194</v>
       </c>
     </row>
     <row r="7">
@@ -12693,7 +12693,7 @@
         <v>0</v>
       </c>
       <c r="Q7" t="n">
-        <v>7.14</v>
+        <v>7.1436</v>
       </c>
     </row>
     <row r="8">
@@ -12712,7 +12712,7 @@
         <v>215786</v>
       </c>
       <c r="E8" t="n">
-        <v>15.53</v>
+        <v>15.5274</v>
       </c>
       <c r="F8" t="n">
         <v>56676</v>
@@ -12748,7 +12748,7 @@
         <v>0</v>
       </c>
       <c r="Q8" t="n">
-        <v>14</v>
+        <v>13.9995</v>
       </c>
     </row>
     <row r="9">
@@ -12767,7 +12767,7 @@
         <v>1452704</v>
       </c>
       <c r="E9" t="n">
-        <v>23.21</v>
+        <v>23.2075</v>
       </c>
       <c r="F9" t="n">
         <v>253811</v>
@@ -12822,7 +12822,7 @@
         <v>137032</v>
       </c>
       <c r="E10" t="n">
-        <v>9.25</v>
+        <v>9.246499999999999</v>
       </c>
       <c r="F10" t="n">
         <v>43094</v>
@@ -12858,7 +12858,7 @@
         <v>0</v>
       </c>
       <c r="Q10" t="n">
-        <v>9.25</v>
+        <v>9.2532</v>
       </c>
     </row>
     <row r="11">
@@ -12877,7 +12877,7 @@
         <v>68278</v>
       </c>
       <c r="E11" t="n">
-        <v>8.029999999999999</v>
+        <v>8.0314</v>
       </c>
       <c r="F11" t="n">
         <v>23355</v>
@@ -12913,7 +12913,7 @@
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>7.41</v>
+        <v>7.4116</v>
       </c>
     </row>
     <row r="12">
@@ -12932,7 +12932,7 @@
         <v>335670</v>
       </c>
       <c r="E12" t="n">
-        <v>14.04</v>
+        <v>14.0387</v>
       </c>
       <c r="F12" t="n">
         <v>89553</v>
@@ -12968,7 +12968,7 @@
         <v>1</v>
       </c>
       <c r="Q12" t="n">
-        <v>12.64</v>
+        <v>12.6409</v>
       </c>
     </row>
     <row r="13">
@@ -13023,7 +13023,7 @@
         <v>0</v>
       </c>
       <c r="Q13" t="n">
-        <v>12.57</v>
+        <v>12.5748</v>
       </c>
     </row>
     <row r="14">
@@ -13042,7 +13042,7 @@
         <v>76907</v>
       </c>
       <c r="E14" t="n">
-        <v>12.51</v>
+        <v>12.5143</v>
       </c>
       <c r="F14" t="n">
         <v>23676</v>
@@ -13078,7 +13078,7 @@
         <v>0</v>
       </c>
       <c r="Q14" t="n">
-        <v>11.8</v>
+        <v>11.7973</v>
       </c>
     </row>
     <row r="15">
@@ -13097,7 +13097,7 @@
         <v>66800</v>
       </c>
       <c r="E15" t="n">
-        <v>13.31</v>
+        <v>13.3136</v>
       </c>
       <c r="F15" t="n">
         <v>18756</v>
@@ -13133,7 +13133,7 @@
         <v>0</v>
       </c>
       <c r="Q15" t="n">
-        <v>11.48</v>
+        <v>11.4764</v>
       </c>
     </row>
     <row r="16">
@@ -13152,7 +13152,7 @@
         <v>150949</v>
       </c>
       <c r="E16" t="n">
-        <v>11.61</v>
+        <v>11.6084</v>
       </c>
       <c r="F16" t="n">
         <v>53016</v>
@@ -13188,7 +13188,7 @@
         <v>0</v>
       </c>
       <c r="Q16" t="n">
-        <v>9.99</v>
+        <v>9.9924</v>
       </c>
     </row>
     <row r="17">
@@ -13207,7 +13207,7 @@
         <v>81468</v>
       </c>
       <c r="E17" t="n">
-        <v>7.96</v>
+        <v>7.9575</v>
       </c>
       <c r="F17" t="n">
         <v>29796</v>
@@ -13243,7 +13243,7 @@
         <v>0</v>
       </c>
       <c r="Q17" t="n">
-        <v>6.76</v>
+        <v>6.7649</v>
       </c>
     </row>
     <row r="18">
@@ -13262,7 +13262,7 @@
         <v>138559</v>
       </c>
       <c r="E18" t="n">
-        <v>10.9</v>
+        <v>10.8984</v>
       </c>
       <c r="F18" t="n">
         <v>34747</v>
@@ -13298,7 +13298,7 @@
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>9.77</v>
+        <v>9.766999999999999</v>
       </c>
     </row>
     <row r="19">
@@ -13317,7 +13317,7 @@
         <v>228956</v>
       </c>
       <c r="E19" t="n">
-        <v>12.26</v>
+        <v>12.2637</v>
       </c>
       <c r="F19" t="n">
         <v>66086</v>
@@ -13353,7 +13353,7 @@
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>10.66</v>
+        <v>10.6587</v>
       </c>
     </row>
     <row r="20">
@@ -13372,7 +13372,7 @@
         <v>50667</v>
       </c>
       <c r="E20" t="n">
-        <v>9.01</v>
+        <v>9.007300000000001</v>
       </c>
       <c r="F20" t="n">
         <v>12856</v>
@@ -13408,7 +13408,7 @@
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>7.21</v>
+        <v>7.2054</v>
       </c>
     </row>
     <row r="21">
@@ -13427,7 +13427,7 @@
         <v>231780</v>
       </c>
       <c r="E21" t="n">
-        <v>12.79</v>
+        <v>12.7891</v>
       </c>
       <c r="F21" t="n">
         <v>70254</v>
@@ -13463,7 +13463,7 @@
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>12.31</v>
+        <v>12.3123</v>
       </c>
     </row>
     <row r="22">
@@ -13482,7 +13482,7 @@
         <v>192702</v>
       </c>
       <c r="E22" t="n">
-        <v>11.64</v>
+        <v>11.6432</v>
       </c>
       <c r="F22" t="n">
         <v>73272</v>
@@ -13518,7 +13518,7 @@
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>10.5</v>
+        <v>10.5026</v>
       </c>
     </row>
     <row r="23">
@@ -13537,7 +13537,7 @@
         <v>71747</v>
       </c>
       <c r="E23" t="n">
-        <v>8.449999999999999</v>
+        <v>8.446199999999999</v>
       </c>
       <c r="F23" t="n">
         <v>29068</v>
@@ -13573,7 +13573,7 @@
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>6.95</v>
+        <v>6.9472</v>
       </c>
     </row>
     <row r="24">
@@ -13592,7 +13592,7 @@
         <v>123000</v>
       </c>
       <c r="E24" t="n">
-        <v>9.119999999999999</v>
+        <v>9.1189</v>
       </c>
       <c r="F24" t="n">
         <v>50099</v>
@@ -13628,7 +13628,7 @@
         <v>5</v>
       </c>
       <c r="Q24" t="n">
-        <v>7.73</v>
+        <v>7.7268</v>
       </c>
     </row>
     <row r="25">
@@ -13647,7 +13647,7 @@
         <v>180235</v>
       </c>
       <c r="E25" t="n">
-        <v>10.65</v>
+        <v>10.6459</v>
       </c>
       <c r="F25" t="n">
         <v>58540</v>
@@ -13683,7 +13683,7 @@
         <v>6</v>
       </c>
       <c r="Q25" t="n">
-        <v>9.81</v>
+        <v>9.813599999999999</v>
       </c>
     </row>
     <row r="26">
@@ -13702,7 +13702,7 @@
         <v>503912</v>
       </c>
       <c r="E26" t="n">
-        <v>18.74</v>
+        <v>18.7389</v>
       </c>
       <c r="F26" t="n">
         <v>146722</v>
@@ -13738,7 +13738,7 @@
         <v>0</v>
       </c>
       <c r="Q26" t="n">
-        <v>17.44</v>
+        <v>17.4415</v>
       </c>
     </row>
     <row r="27">
@@ -13757,7 +13757,7 @@
         <v>65335</v>
       </c>
       <c r="E27" t="n">
-        <v>7.76</v>
+        <v>7.7569</v>
       </c>
       <c r="F27" t="n">
         <v>27647</v>
@@ -13793,7 +13793,7 @@
         <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>5.95</v>
+        <v>5.9474</v>
       </c>
     </row>
     <row r="28">
@@ -13812,7 +13812,7 @@
         <v>34934</v>
       </c>
       <c r="E28" t="n">
-        <v>7.44</v>
+        <v>7.4409</v>
       </c>
       <c r="F28" t="n">
         <v>13906</v>
@@ -13848,7 +13848,7 @@
         <v>0</v>
       </c>
       <c r="Q28" t="n">
-        <v>6.41</v>
+        <v>6.413</v>
       </c>
     </row>
     <row r="29">
@@ -13867,7 +13867,7 @@
         <v>215180</v>
       </c>
       <c r="E29" t="n">
-        <v>16.42</v>
+        <v>16.4184</v>
       </c>
       <c r="F29" t="n">
         <v>68107</v>
@@ -13903,7 +13903,7 @@
         <v>0</v>
       </c>
       <c r="Q29" t="n">
-        <v>15.86</v>
+        <v>15.8561</v>
       </c>
     </row>
     <row r="30">
@@ -13922,7 +13922,7 @@
         <v>1250319</v>
       </c>
       <c r="E30" t="n">
-        <v>25.66</v>
+        <v>25.6554</v>
       </c>
       <c r="F30" t="n">
         <v>147133</v>
@@ -13958,7 +13958,7 @@
         <v>5</v>
       </c>
       <c r="Q30" t="n">
-        <v>25.33</v>
+        <v>25.3302</v>
       </c>
     </row>
     <row r="31">
@@ -13977,7 +13977,7 @@
         <v>40926</v>
       </c>
       <c r="E31" t="n">
-        <v>7.94</v>
+        <v>7.9407</v>
       </c>
       <c r="F31" t="n">
         <v>15917</v>
@@ -14013,7 +14013,7 @@
         <v>0</v>
       </c>
       <c r="Q31" t="n">
-        <v>6.93</v>
+        <v>6.9327</v>
       </c>
     </row>
     <row r="32">
@@ -14032,7 +14032,7 @@
         <v>11121</v>
       </c>
       <c r="E32" t="n">
-        <v>5.51</v>
+        <v>5.5141</v>
       </c>
       <c r="F32" t="n">
         <v>3963</v>
@@ -14068,7 +14068,7 @@
         <v>0</v>
       </c>
       <c r="Q32" t="n">
-        <v>3.49</v>
+        <v>3.4852</v>
       </c>
     </row>
     <row r="33">
@@ -14087,7 +14087,7 @@
         <v>136563</v>
       </c>
       <c r="E33" t="n">
-        <v>12.46</v>
+        <v>12.4613</v>
       </c>
       <c r="F33" t="n">
         <v>44202</v>
@@ -14123,7 +14123,7 @@
         <v>7</v>
       </c>
       <c r="Q33" t="n">
-        <v>11.83</v>
+        <v>11.8322</v>
       </c>
     </row>
     <row r="34">
@@ -14142,7 +14142,7 @@
         <v>226397</v>
       </c>
       <c r="E34" t="n">
-        <v>16.34</v>
+        <v>16.3404</v>
       </c>
       <c r="F34" t="n">
         <v>47227</v>
@@ -14178,7 +14178,7 @@
         <v>0</v>
       </c>
       <c r="Q34" t="n">
-        <v>16</v>
+        <v>16.0013</v>
       </c>
     </row>
   </sheetData>

</xml_diff>